<commit_message>
docs(nidp): update feed inventory — 5 new feeds, NSE_FINANCIALS 3-strategy pipeline; add PRD v2 + Rule Book
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/NIDP_FEEDS/Master_Data_Feed_Template.xlsx
+++ b/docs/NIDP_FEEDS/Master_Data_Feed_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Feed Inventory" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Scoring &amp; Derived Tables" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Tasks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feed Inventory" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring &amp; Derived Tables" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Tasks'!$A$4:$M$29</definedName>
@@ -854,7 +854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AB40"/>
+  <dimension ref="A1:AB45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="9" min="1" max="2"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="N12" s="17" t="inlineStr">
         <is>
-          <t>NSE (primary XBRL); company IR pages (fallback scrape + LLM extract)</t>
+          <t>NSE corporate-announcements API (primary XBRL _WEB.xml); company IR pages via company_ir_urls table (secondary scrape); NSE XBRL comparator API (tertiary JSON)</t>
         </is>
       </c>
       <c r="O12" s="17" t="inlineStr">
@@ -2419,7 +2419,12 @@
       </c>
       <c r="U12" s="17" t="inlineStr">
         <is>
-          <t>GET list → per filing: try company IR page first (scrape + Claude LLM extraction) → fallback to NSE XBRL comparator → parse XBRL namespace-agnostic by local-name → emit standalone + consolidated rows if both present → scale ₹ to crores → COALESCE upsert.</t>
+          <t>3-strategy pipeline per company:
+1) NSE Integrated XBRL filing (_WEB.xml via corporate-announcements API) — zero LLM tokens, reads IndAS/IGAAP contextRef='OneD' P&amp;L + 'OneI' balance sheet
+2) Company IR page (ir_url from company_ir_urls) — scrape HTML/PDF, extract text (pdfminer for PDFs), pass to LLM if not XML
+3) NSE XBRL comparator API (JSON) — parse JSON directly, LLM fallback
+LLM backend: OPENAI_API_KEY → gpt-4o-mini; else ANTHROPIC_API_KEY → claude-haiku-4-5
+period_end inferred from event_date if LLM returns null</t>
         </is>
       </c>
       <c r="V12" s="17" t="inlineStr">
@@ -2454,7 +2459,9 @@
       </c>
       <c r="AB12" s="17" t="inlineStr">
         <is>
-          <t>15d: 19 OK / 0 FAILED. FLAG: LLM fallback (Claude Haiku) means quiet API-key dependency; failure mode if ANTHROPIC_API_KEY rotates without redeploy.</t>
+          <t>Updated 2026-05-26: 3-strategy pipeline with NSE Integrated XBRL as primary (no LLM).
+OpenAI gpt-4o-mini added as primary LLM backend (Anthropic Haiku fallback).
+15d: 19 OK / 0 FAILED. FLAG: LLM fallback means quiet API-key dependency; OPENAI_API_KEY must be set in nidp.env. Source run_id written per upsert for dedup tracing.</t>
         </is>
       </c>
     </row>
@@ -6431,6 +6438,566 @@
       <c r="AB40" s="19" t="inlineStr">
         <is>
           <t>15d: 4 OK / 141 FAILED. **CRITICAL**: failure is NotFound 404 on gs://nidp-raw-niveshdataintelligence/portfolio/holdings/2025-07-31/holdings.jsonl. The upstream Nivesh portfolio_gcs_export is either NOT writing files OR writing to a different bucket/path. 141 failures = run scheduled but file never lands. Investigate Nivesh app's export job.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Feed 38</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>V3_SCORES_ENGINE</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>v3_scores_engine</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Linux cron (/etc/cron.d/nidp)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>23:55 IST (Mon-Fri)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Daily (trading days)</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>55 23 * * 1-5  (IST)</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Time-based</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Computes and persists V3 composite Quality + Health scores for every MF scheme and NSE stock. Writes nightly snapshot rows to nidp.v3_mf_scores_daily and nidp.v3_stock_scores_daily.</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Derived scoring: Quality score (0-100), Health score (0-100) per MF/stock. Served by /v1/{mf,stocks}/scores/*.</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Internal derived</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>TimescaleDB: nidp.mf_derived_analytics, nidp.stock_features_daily, nidp.technical_indicators</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>nidp.v3_mf_scores_daily  •  nidp.v3_stock_scores_daily</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Postgres 16 + TimescaleDB (nidp-postgres, db: nidp)</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Insert with date partition; idempotent via ON CONFLICT (date, isin/symbol)</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>backend/nidp/services/v3_scores_engine/</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>mf_derived_refresh (23:50)  •  fundamental_engine (23:05)  •  technical_indicator_engine (22:35)</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>Nivesh portfolio health scoring  •  /api/insights/v3-portfolio  •  intelligence_layer</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>~2-5 min</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Grafana NIDP Feed Schedule and Status</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>Idempotent. Manual: sudo -u nidp run_service.sh v3_scores_engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Feed 39</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ANALYTICS_REFRESH</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>analytics_refresh</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Linux cron (/etc/cron.d/nidp)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>00:10 IST (Tue-Sat, i.e. after Mon-Fri trading sessions)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Daily (trading days + 1)</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>10 0 * * 2-6  (IST)</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Time-based</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Populates analytics.stock_card + analytics.sector_snapshot and refreshes 4 materialized views: mv_top_momentum, mv_delivery_surge, mv_sector_heatmap, mv_fund_category_top10.</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Derived analytics: momentum, delivery surge, sector heatmap, fund category rankings</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Internal derived</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>TimescaleDB: nidp.bhavcopy, nidp.delivery, nidp.stock_features_daily, nidp.v3_stock_scores_daily</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>analytics.stock_card  •  analytics.sector_snapshot  •  analytics.mv_top_momentum  •  analytics.mv_delivery_surge  •  analytics.mv_sector_heatmap  •  analytics.mv_fund_category_top10</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Postgres 16 + TimescaleDB (nidp-postgres, db: nidp)</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Upsert + REFRESH MATERIALIZED VIEW CONCURRENTLY</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>backend/nidp/services/analytics_refresh/</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>v3_scores_engine (23:55)  •  snapshot_builder (22:00)  •  technical_indicator_engine (22:35)</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>DaaS API analytics endpoints  •  market intelligence feeds</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>~3-8 min</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>Grafana NIDP Feed Schedule and Status</t>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>Idempotent REFRESH + upsert. Manual: sudo -u nidp run_service.sh analytics_refresh</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Feed 40</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>PORTFOLIO_TRANSACTIONS_SYNC</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>portfolio_transactions_sync</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Linux cron (/etc/cron.d/nidp)</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>23:10 IST (Mon-Fri)</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Daily (trading days)</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>10 23 * * 1-5  (IST)</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Time-based</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Reads per-user transaction JSONL exports from GCS and upserts into portfolio.user_transactions_snapshot. Runs after portfolio_holdings_sync to ensure client_master rows exist.</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Per-user transactions: buy/sell/switch/dividend history. PII.</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Internal (per-user PII)</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>GCS landing zone: gs://{NIDP_GCS_BUCKET}/portfolio/transactions/{date}/transactions.jsonl</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>portfolio.user_transactions_snapshot</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Postgres 16 + TimescaleDB (nidp-postgres, db: nidp)</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Upsert with dedup hash</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>backend/nidp/services/portfolio_transactions_sync/</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>portfolio_holdings_sync (23:00) — must succeed first</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>portfolio_intelligence_sync  •  tax engine  •  performance analytics</t>
+        </is>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>Grafana NIDP Feed Schedule and Status</t>
+        </is>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>Idempotent. Manual: sudo -u nidp run_service.sh portfolio_transactions_sync</t>
+        </is>
+      </c>
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>BLOCKED by portfolio_holdings_sync GCS 404 failure. Fix GCS export in Nivesh app first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Feed 41</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>PORTFOLIO_GOALS_SYNC</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>portfolio_goals_sync</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Linux cron (/etc/cron.d/nidp)</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>23:15 IST (Mon-Fri)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Daily (trading days)</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>15 23 * * 1-5  (IST)</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Time-based</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Syncs per-user goal definitions from Nivesh PG (user_goals) to NIDP so the intelligence_layer can evaluate goal alignment and compute on_track_pct.</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Per-user goals: target amount, horizon, current corpus, SIP, on-track %. PII.</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Internal (per-user PII)</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Nivesh Postgres: user_goals table (GCS or direct PG bridge)</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>portfolio.user_goals_snapshot</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Postgres 16 + TimescaleDB (nidp-postgres, db: nidp)</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Upsert</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>backend/nidp/services/portfolio_goals_sync/</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>portfolio_holdings_sync (23:00)  •  portfolio_transactions_sync (23:10)</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>intelligence_layer (23:20)  •  portfolio_intelligence_sync (23:30)  •  Goal Alignment Engine</t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>Grafana NIDP Feed Schedule and Status</t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>Idempotent. Manual: sudo -u nidp run_service.sh portfolio_goals_sync</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Feed 42</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>AMC_URLS_DRIFT_CHECK</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>amc_urls_drift_check</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>PROD</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Linux cron (/etc/cron.d/nidp)</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>08:00 IST daily</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>0 8 * * *  (IST)</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Time-based</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Daily health check that pings every AMC website + AMFI listing candidate URL. Marks JobRun FAILED if any AMC has zero healthy URL candidates — enables early detection of URL rot for mf_disclosure_snapshot and mf_holdings.</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Health check / URL liveness. No data ingested.</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Internal operational</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>HTTP pings to ~10 AMC websites (HDFC, ICICI, SBI, Axis, Kotak, Nippon, etc.)</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>nidp.job_log (status only)</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Postgres 16 + TimescaleDB (nidp-postgres, db: nidp)</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Status write only (no data rows)</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>backend/nidp/services/amc_urls_drift_check/</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>None (independent sentinel)</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>Alerting / Grafana  •  Indirectly: mf_disclosure_snapshot + mf_holdings depend on healthy URLs</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>~30-60 sec</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>Grafana NIDP Feed Schedule and Status. FAILED = at least one AMC URL is broken.</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>Fix AMC URL in config/seed data. Manual: sudo -u nidp run_service.sh amc_urls_drift_check</t>
+        </is>
+      </c>
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>Currently all 10 AMC scraper URLs are 404 or changed. This check should be alerting daily. See open_bugs.md: AMC scrapers all broken.</t>
         </is>
       </c>
     </row>

</xml_diff>